<commit_message>
feat: 6 semester-specific weight sets + Set_ID selector + sorted bar charts
</commit_message>
<xml_diff>
--- a/data/Plantilla_V4_Refinada.xlsx
+++ b/data/Plantilla_V4_Refinada.xlsx
@@ -26,7 +26,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Oferta_x_Programa'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Calidad'!$A$1:$T$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Costo_del_Sitio'!$A$1:$K$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Ponderaciones'!$A$5:$L$16</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,35 +473,6 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Ricardo Alberto Arango Cardona</author>
-  </authors>
-  <commentList>
-    <comment ref="B2" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-   El set corresponde a un conjunto de reglas que aplique para un programa determinado. El set001 es de ejemplo, se puede crear setMedicina con las reglas especificas y de interés para medicina o para cualquier programa de interés.
-</t>
-      </text>
-    </comment>
-    <comment ref="I5" authorId="0" shapeId="0">
-      <text>
-        <t>Los pesos (Activos) del mismo Set_ID deben sumar 1.00.</t>
-      </text>
-    </comment>
-    <comment ref="L5" authorId="0" shapeId="0">
-      <text>
-        <t>Auto: suma de pesos (I) donde Set_ID coincide y Activo=1.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -21120,148 +21090,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81428571428571" defaultRowHeight="14.5"/>
+  <dimension ref="A1:L65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" style="18" min="1" max="1"/>
+    <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="35" customWidth="1" style="18" min="2" max="2"/>
     <col width="28" customWidth="1" style="18" min="3" max="3"/>
     <col width="21" customWidth="1" style="18" min="4" max="4"/>
-    <col width="44" customWidth="1" style="18" min="5" max="5"/>
+    <col width="28" customWidth="1" style="18" min="5" max="5"/>
     <col width="26" customWidth="1" style="18" min="6" max="6"/>
-    <col width="42" customWidth="1" style="18" min="7" max="7"/>
+    <col width="35" customWidth="1" style="18" min="7" max="7"/>
     <col width="24" customWidth="1" style="18" min="8" max="8"/>
     <col width="12" customWidth="1" style="18" min="9" max="9"/>
     <col width="14" customWidth="1" style="18" min="10" max="10"/>
-    <col width="12" customWidth="1" style="18" min="11" max="11"/>
+    <col width="35" customWidth="1" style="18" min="11" max="11"/>
     <col width="35" customWidth="1" style="18" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5" customHeight="1" s="18">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>CONTROL DEL SET (para validar que la suma de pesos activos sea 1.00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14.5" customHeight="1" s="18">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Set_ID a validar:</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SET001</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo:</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" ht="14.5" customHeight="1" s="18">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Suma pesos activos (de ese Set_ID):</t>
-        </is>
-      </c>
-      <c r="B3" s="3">
-        <f>SUMIFS($I:$I,$A:$A,$B$2,$J:$J,1)</f>
-        <v/>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Estado:</t>
-        </is>
-      </c>
-      <c r="E3">
-        <f>IF(ABS($B$3-1)&lt;=0.0001,"OK","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" ht="14.5" customHeight="1" s="18">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Nota: Solo se suman los pesos con Activo=1. La suma debe dar 1.00.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1" s="18">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Set_ID</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Nombre_Set</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Semestre_Vigencia (AAAA-S)</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Programa (o GLOBAL)</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Tipo_Estudiante (opcional)</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Tipo_Practica (opcional)</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Criterio_Codigo</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Tipo (Beneficio/Costo)</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>Peso (0-1)</t>
         </is>
       </c>
-      <c r="J5" s="1" t="inlineStr">
+      <c r="J5" s="22" t="inlineStr">
         <is>
           <t>Activo (0/1)</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="L5" s="1" t="inlineStr">
+      <c r="L5" s="22" t="inlineStr">
         <is>
           <t>Suma_Pesos_Activos_del_Set (auto)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="14.5" customHeight="1" s="18">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SET-MEDICINA</t>
+          <t>SET-SEM5-SaludPublica</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ponderación Medicina</t>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21289,500 +21209,2852 @@
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Escenario_Avalado_Practicas</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Servicios_Pediatricos (0/1)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SET-SEM5-SaludPublica</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sem 5 - Salud Pública y Comunidad</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, hospitales universitarios y escenarios avalados</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Es_Hospital_Universitario</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Escenario_Avalado_Practicas</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Servicios_Pediatricos (0/1)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>0.1</v>
       </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <f>SUMIFS($I:$I,$A:$A,$A6,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" s="18">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>2026-1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Pregrado</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SET-SEM6-Psiquiatria</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sem 6 - Psiquiatría y Enlace</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con evaluación, docentes externos, áreas académicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Es_Hospital_Universitario</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>Escenario_Avalado_Practicas</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Servicios_Pediatricos (0/1)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SET-SEM7-MedicinaInterna</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sem 7 - Medicina Interna y Especialidades</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con vinculación de especialistas, evaluación, académicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Es_Hospital_Universitario</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Escenario_Avalado_Practicas</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Servicios_Pediatricos (0/1)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SET-SEM8-Pediatria</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sem 8 - Pediatría</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con servicios pediátricos, obstetricia, bienestar</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Es_Hospital_Universitario</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Escenario_Avalado_Practicas</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Servicios_Pediatricos (0/1)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SET-SEM9-Gineco</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Sem 9 - Ginecobstetricia y Urgencias</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con obstetricia, quirófanos, urgencias, bajo costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Es_Hospital_Universitario</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
         <v>0.2</v>
       </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <f>SUMIFS($I:$I,$A:$A,$A7,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="14.5" customHeight="1" s="18">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
         <is>
           <t>2026-1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Pregrado</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Escenario_Avalado_Practicas</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
         <is>
           <t>Servicios_Pediatricos (0/1)</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Servicios_Obstetricia (0/1)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
         <v>0.1</v>
       </c>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8">
-        <f>SUMIFS($I:$I,$A:$A,$A8,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="14.5" customHeight="1" s="18">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
         <is>
           <t>2026-1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Pregrado</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Servicios_Obstetricia (0/1)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
         <is>
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I9" s="16" t="n">
+      <c r="I60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Admiten_Docentes_Externos (Sí/No)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Beneficio</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
         <v>0.1</v>
       </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9">
-        <f>SUMIFS($I:$I,$A:$A,$A9,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="14.5" customHeight="1" s="18">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t>2026-1</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Pregrado</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>MisionVisionProposito_AlineacionDocencia (1-5)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Areas_Bienestar (0/1)</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I10" s="16" t="n">
+      <c r="I62" t="n">
         <v>0.05</v>
       </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10">
-        <f>SUMIFS($I:$I,$A:$A,$A10,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="14.5" customHeight="1" s="18">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
         <is>
           <t>2026-1</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Pregrado</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Admiten_Docentes_Externos (Sí/No)</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Areas_Academicas (0/1)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
         <is>
           <t>Beneficio</t>
         </is>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I63" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>%_Contraprestacion_Matricula (0-100)</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SET-SEM10-Cirugia</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Sem 10 - Cirugía y Urgencias</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Pregrado</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
         <v>0.05</v>
       </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11">
-        <f>SUMIFS($I:$I,$A:$A,$A11,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="14.5" customHeight="1" s="18">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-1</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Medicina</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Pregrado</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Areas_Bienestar (0/1)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Beneficio</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12">
-        <f>SUMIFS($I:$I,$A:$A,$A12,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="14.5" customHeight="1" s="18">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Medicina</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Pregrado</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Areas_Academicas (0/1)</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Beneficio</t>
-        </is>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13">
-        <f>SUMIFS($I:$I,$A:$A,$A13,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="14.5" customHeight="1" s="18">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medicina</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Pregrado</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>%_Contraprestacion_Matricula (0-100)</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Costo</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14">
-        <f>SUMIFS($I:$I,$A:$A,$A14,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="14.5" customHeight="1" s="18">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2026-1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medicina</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Pregrado</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>EPP_Exigidos (Sin exigencia/Parcial/Completo + detalle)</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Costo</t>
-        </is>
-      </c>
-      <c r="I15" s="16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15">
-        <f>SUMIFS($I:$I,$A:$A,$A15,$J:$J,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="14.5" customHeight="1" s="18">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SET-MEDICINA</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Ponderación Medicina</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medicina</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Pregrado</t>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Prioriza IPS con quirófanos, especialistas, menor costo, medicina de urgencias</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:L16"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="expression" priority="6" dxfId="3">
-      <formula>ABS($B$3-1)&gt;0.0001</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="4">
-      <formula>ABS($B$3-1)&lt;=0.0001</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L6:L500">
-    <cfRule type="expression" priority="4" dxfId="3">
-      <formula>AND($A6&lt;&gt;"",ABS(L6-1)&gt;0.0001)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="H6:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Beneficio,Costo"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J6:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"0,1"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I6:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Validación" error="Valor inválido. Debe estar entre 0 y 1." type="decimal">
-      <formula1>0</formula1>
-      <formula2>1</formula2>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add temporal component (MVP) with 08_Calendario, TemporalGroupOptimizer, and calendar visualization in app
</commit_message>
<xml_diff>
--- a/data/Plantilla_V4_Refinada.xlsx
+++ b/data/Plantilla_V4_Refinada.xlsx
@@ -15,10 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_Guia_llenado" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Rotaciones" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Demanda_Semestres" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Calendario" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Catalogos'!$A$1:$B$58</definedName>
@@ -13627,6 +13628,1110 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" style="18" min="1" max="1"/>
+    <col width="19" customWidth="1" style="18" min="2" max="2"/>
+    <col width="12" customWidth="1" style="18" min="3" max="3"/>
+    <col width="13" customWidth="1" style="18" min="4" max="4"/>
+    <col width="13" customWidth="1" style="18" min="5" max="5"/>
+    <col width="14" customWidth="1" style="18" min="6" max="6"/>
+    <col width="12" customWidth="1" style="18" min="7" max="7"/>
+    <col width="12" customWidth="1" style="18" min="8" max="8"/>
+    <col width="35" customWidth="1" style="18" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>Semestre_Plan</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>Asignatura</t>
+        </is>
+      </c>
+      <c r="C1" s="22" t="inlineStr">
+        <is>
+          <t>Rotacion</t>
+        </is>
+      </c>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>Tipo_Tiempo</t>
+        </is>
+      </c>
+      <c r="E1" s="22" t="inlineStr">
+        <is>
+          <t>Periodo_Num</t>
+        </is>
+      </c>
+      <c r="F1" s="22" t="inlineStr">
+        <is>
+          <t>Fecha_Inicio</t>
+        </is>
+      </c>
+      <c r="G1" s="22" t="inlineStr">
+        <is>
+          <t>Fecha_Fin</t>
+        </is>
+      </c>
+      <c r="H1" s="22" t="inlineStr">
+        <is>
+          <t>Origen</t>
+        </is>
+      </c>
+      <c r="I1" s="22" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Práctica 1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Práctica 2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Práctica 3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Salud Pública III</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Práctica 4</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>simultanea</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Grupos rotan cada mes entre las 4 prácticas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>